<commit_message>
aicore: On-Prem üstünlükleri sayfası + AICORE Cloud Ready paketi + fiyat duruşu notu
- /aicore/on-prem: On-Prem Yapay Zekâ satış sayfası (6 üstünlük kartı +
  On-Prem vs Maskeli Bulut karşılaştırma tablosu)
- setup/aicore-cloud-ready (SCAICRCP): Maskeli Bulut kurulum paketi —
  GPU'suz altyapı, denetlenebilir maskeleme katmanı, kalibrasyon,
  token maliyeti müşterinin notu, On-Prem'e geçiş yolu
- /aicore vitrini: "Neden On-Prem?" linki + hizmet bölümü 3 karta çıktı
- CRM listesi: Cloud Ready hizmet satırı eklendi (3 hizmet)
- gorevler/ekler: On-Prem/Cloud fiyat duruşu notu (md + txt)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
+++ b/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1027,15 +1027,32 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>AICORE Cloud Ready Paketi</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Maskeli Bulut modunda AICore kurulum hizmeti. Kurum ortamına dil modeli kurulmaz; GPU'suz hafif uygulama sunucusu, kişisel verileri denetlenebilir şekilde maskeleyen katman, kalibrasyon ve eğitimle 1-2 haftada devreye alma. Bulut kullanım (token) maliyeti kurumun kendi API hesabına aittir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-cloud-ready</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>SCAICRCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>AICORE Destek Paketleri</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>AICore eklentileri için Silver, Gold ve Platinum yıllık bakım paketleri. Sürüm güncellemeleri, her güncelleme sonrası otomatik doğrulama koşusu ve periyodik yeniden kalibrasyon tek abonelikte. Yapay zekânın yalnızca çalışır değil, isabetli kalması güvence altına alınır. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>SCAIDSP</t>
         </is>

</xml_diff>

<commit_message>
crm: ağırlıklandırma tablosuna kurulum ve destek hizmeti çarpanları eklendi
Modül başına üç ayrı çarpan: Lisans (değer ağırlıklı) + Kurulum Hizmeti
(kurulum zorluğu ekseni) + Destek Hizmeti (bakım zorluğu ekseni).
Formüller tablonun altında.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
+++ b/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1078,7 +1078,9 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1109,10 +1111,20 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Fiyat Çarpanı</t>
+          <t>Lisans Çarpanı</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Kurulum Hizmeti Çarpanı</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Destek Hizmeti Çarpanı</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Gerekçe</t>
         </is>
@@ -1143,7 +1155,17 @@
           <t>3.2X</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>5.0X</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Son kullanıcıya açık: kanal entegrasyonu + yüksek eşzamanlılık</t>
         </is>
@@ -1174,7 +1196,17 @@
           <t>3.0X</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Amiral gemisi; kalibrasyon + geri bildirim döngüsü bakım ister</t>
         </is>
@@ -1205,7 +1237,17 @@
           <t>2.9X</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Yüksek değer (bilgi bankası otomasyonu); kurulum + onay akışı kapsamlı</t>
         </is>
@@ -1236,7 +1278,17 @@
           <t>2.9X</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>5.0X</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Ağ keşfi: kurum BT'siyle ortak kurulum, en ağırlardan</t>
         </is>
@@ -1267,7 +1319,17 @@
           <t>2.9X</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>5.0X</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Santral entegrasyonu + konuşma tanıma; ağır kurulum</t>
         </is>
@@ -1298,7 +1360,17 @@
           <t>2.7X</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Zafiyet verisi güncelleme bakımı sürekli</t>
         </is>
@@ -1329,7 +1401,17 @@
           <t>2.5X</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Öğrenme döngüsü sürekli izleme/bakım ister</t>
         </is>
@@ -1360,7 +1442,17 @@
           <t>2.5X</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Alarm sistemleri entegrasyonu + tepe hacim</t>
         </is>
@@ -1391,7 +1483,17 @@
           <t>2.5X</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Ses akışı + kayıt depolama</t>
         </is>
@@ -1422,7 +1524,17 @@
           <t>2.3X</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Doküman kaynak erişimi kurulumu; işleme hattı ortak</t>
         </is>
@@ -1453,7 +1565,17 @@
           <t>2.3X</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Kategori/atama eğitimi + müşteri şemasına uyarlama</t>
         </is>
@@ -1484,7 +1606,17 @@
           <t>2.3X</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Tahmin kalitesi izleme ister</t>
         </is>
@@ -1515,7 +1647,17 @@
           <t>2.2X</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Yönetici görünürlüğü yüksek; rapor şemasına uyarlama</t>
         </is>
@@ -1546,7 +1688,17 @@
           <t>2.0X</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Yüksek görünür değer; teknik olarak hafif</t>
         </is>
@@ -1577,7 +1729,17 @@
           <t>2.0X</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Telemetri kaynaklarına bağımlı</t>
         </is>
@@ -1608,7 +1770,17 @@
           <t>1.9X</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Varlık ilişkisi verisine bağımlı</t>
         </is>
@@ -1639,7 +1811,17 @@
           <t>1.9X</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Yapılandırma düzeyi yazma; onay akışı şart</t>
         </is>
@@ -1670,7 +1852,17 @@
           <t>1.9X</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>İK/vardiya verisi entegrasyonu</t>
         </is>
@@ -1701,7 +1893,17 @@
           <t>1.9X</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Periyodik denetim; orta kapsam</t>
         </is>
@@ -1732,7 +1934,17 @@
           <t>1.9X</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Finans verisi entegrasyonu</t>
         </is>
@@ -1763,7 +1975,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Motor hazır; sınırlı yüzey</t>
         </is>
@@ -1794,7 +2016,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Dar kapsam, hafif</t>
         </is>
@@ -1825,7 +2057,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Bilgi bankası taraması; orta kapsam</t>
         </is>
@@ -1856,7 +2098,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Görsel okuma; mevcut yeteneğin ürünleşmesi</t>
         </is>
@@ -1887,7 +2139,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Doküman deposu erişimi; orta</t>
         </is>
@@ -1918,7 +2180,17 @@
           <t>1.7X</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Proje verisi analizi; orta</t>
         </is>
@@ -1949,7 +2221,17 @@
           <t>1.3X</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Dar kapsam</t>
         </is>
@@ -1980,7 +2262,17 @@
           <t>1.3X</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>2.0X</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Dar kapsam</t>
         </is>
@@ -2011,7 +2303,17 @@
           <t>1.0X</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Basit analiz; taban ürün</t>
         </is>
@@ -2042,7 +2344,17 @@
           <t>1.0X</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Basit analiz; taban ürün</t>
         </is>
@@ -2073,7 +2385,17 @@
           <t>1.0X</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Basit çeviri katmanı; taban ürün</t>
         </is>
@@ -2082,7 +2404,28 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Model: çarpan = (0,5·Değer + 0,3·Kurulum + 0,2·Bakım) / taban. En hafif ürün 1.0X kabul edilir; fiyat = taban fiyat × çarpan.</t>
+          <t>Model — üç ayrı çarpan, üç ayrı fiyat kalemi:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>· Lisans Çarpanı = (0,5·Değer + 0,3·Kurulum + 0,2·Bakım) / taban → modül lisans fiyatı = lisans tabanı × bu çarpan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>· Kurulum Hizmeti Çarpanı = Kurulum Zorluğu / taban → modül kurulum bedeli = kurulum tabanı (Launch Ready veya Cloud Ready) × bu çarpan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>· Destek Hizmeti Çarpanı = Bakım Zorluğu / taban → modülün yıllık destek payı = destek tabanı (Silver/Gold/Platinum) × bu çarpan; sözleşme tek, fiyat toplamdan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
aicore-destek: 4 paket + karşılaştırma tablosu (SM destek paketleri paralel)
- Silver/Gold/Platinum/Mission Critical — kodlar CRM ile birebir
  (SCAISSP/SCAIGSP/SCAIPSP/SCAIMCSP)
- 16 satırlık karşılaştırma tablosu: ticket hakkı (15/30/60/60), çalışma
  saatleri (5x8→7x24), kanallar + AI'a özgü satırlar (kalibrasyon,
  oto-doğrulama, sağlık raporu, AI Health-Check, adanmış uzman)
- 4 paket konumlama kartı (comparison bölümü)
- CRM listesi: tek destek satırı → 4 ayrı paket satırı

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
+++ b/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1044,17 +1044,68 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AICORE Destek Paketleri</t>
+          <t>AICORE Silver Destek Paketi</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>AICore eklentileri için Silver, Gold ve Platinum yıllık bakım paketleri. Sürüm güncellemeleri, her güncelleme sonrası otomatik doğrulama koşusu ve periyodik yeniden kalibrasyon tek abonelikte. Yapay zekânın yalnızca çalışır değil, isabetli kalması güvence altına alınır. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>AICore eklentileri için temel yıllık bakım. Yıllık 15 ticket, 5x8 kapsam, sürüm güncellemeleri + güncelleme sonrası otomatik doğrulama, yılda 1 yeniden kalibrasyon ve yıllık sağlık raporu. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SCAIDSP</t>
+          <t>SCAISSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AICORE Gold Destek Paketi</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Birden çok AICore eklentisi kullanan kurumlar için yıllık bakım. Yıllık 30 ticket, 5x8 kapsam + telefon desteği, yılda 2 yeniden kalibrasyon, çeyreklik sağlık raporu ve AI Health-Check. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>SCAIGSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>AICORE Platinum Destek Paketi</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zekâyı iş akışının parçası yapmış kurumlar için yıllık bakım. Yıllık 60 ticket, 7x8 kapsam + anlık mesaj, yılda 4 yeniden kalibrasyon, aylık sağlık raporu, yüksek öncelikli müdahale ve model performansı izleme. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>SCAIPSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>AICORE Mission Critical Destek Paketi</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zekâsı kesintiye tahammülü olmayan kurumlar için en üst kademe. Yıllık 60 ticket, 7x24 kesintisiz kapsam, sınırsız yeniden kalibrasyon, aylık rapor + dönemsel değerlendirme ve adanmış yapay zekâ uzmanı. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SCAIMCSP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hizmetler: AICORE Quick Start Konfigürasyon Paketi (SCAIQSCP)
Model: ilk kurulum Launch Ready/Cloud Ready (müşteri başına bir kez),
sonraki her add-on Quick Start (eklenti başına).

- setup/aicore-quick-start: zengin sayfa — 5 günlük timeline, 4 aşama,
  Launch Ready fark tablosu, DocCore-ekleme örnekli teslimat panosu
- Launch Ready "sonraki eklentiler" kutusu Quick Start'a bağlandı
- /aicore vitrini hizmet bölümü 4 karta çıktı
- CRM listesi: SCAIQSCP satırı (7 hizmet: LR + CR + QS + 4 destek)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
+++ b/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1044,66 +1044,83 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AICORE Silver Destek Paketi</t>
+          <t>AICORE Quick Start Konfigürasyon Paketi</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>AICore eklentileri için temel yıllık bakım. Yıllık 15 ticket, 5x8 kapsam, sürüm güncellemeleri + güncelleme sonrası otomatik doğrulama, yılda 1 yeniden kalibrasyon ve yıllık sağlık raporu. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>Mevcut AICore altyapısına sonraki her eklentinin devreye alma paketi. Altyapı işi tekrarlanmaz: eklenti kurulumu, varsa ek erişimlerin bağlanması, eklentiye özel kalibrasyon, doğrulama setinin genişletilmesi ve odaklı eğitim — tipik 2-5 gün. İlk kurulum Launch Ready/Cloud Ready ile yapılır; sonraki her eklenti Quick Start ile eklenir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-quick-start</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SCAISSP</t>
+          <t>SCAIQSCP</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AICORE Gold Destek Paketi</t>
+          <t>AICORE Silver Destek Paketi</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Birden çok AICore eklentisi kullanan kurumlar için yıllık bakım. Yıllık 30 ticket, 5x8 kapsam + telefon desteği, yılda 2 yeniden kalibrasyon, çeyreklik sağlık raporu ve AI Health-Check. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>AICore eklentileri için temel yıllık bakım. Yıllık 15 ticket, 5x8 kapsam, sürüm güncellemeleri + güncelleme sonrası otomatik doğrulama, yılda 1 yeniden kalibrasyon ve yıllık sağlık raporu. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SCAIGSP</t>
+          <t>SCAISSP</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AICORE Platinum Destek Paketi</t>
+          <t>AICORE Gold Destek Paketi</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Yapay zekâyı iş akışının parçası yapmış kurumlar için yıllık bakım. Yıllık 60 ticket, 7x8 kapsam + anlık mesaj, yılda 4 yeniden kalibrasyon, aylık sağlık raporu, yüksek öncelikli müdahale ve model performansı izleme. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>Birden çok AICore eklentisi kullanan kurumlar için yıllık bakım. Yıllık 30 ticket, 5x8 kapsam + telefon desteği, yılda 2 yeniden kalibrasyon, çeyreklik sağlık raporu ve AI Health-Check. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SCAIPSP</t>
+          <t>SCAIGSP</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>AICORE Platinum Destek Paketi</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zekâyı iş akışının parçası yapmış kurumlar için yıllık bakım. Yıllık 60 ticket, 7x8 kapsam + anlık mesaj, yılda 4 yeniden kalibrasyon, aylık sağlık raporu, yüksek öncelikli müdahale ve model performansı izleme. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SCAIPSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>AICORE Mission Critical Destek Paketi</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Yapay zekâsı kesintiye tahammülü olmayan kurumlar için en üst kademe. Yıllık 60 ticket, 7x24 kesintisiz kapsam, sınırsız yeniden kalibrasyon, aylık rapor + dönemsel değerlendirme ve adanmış yapay zekâ uzmanı. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>SCAIMCSP</t>
         </is>

</xml_diff>

<commit_message>
aicore: GateCoreAI beta kartı + savunma stratejisi evrakları
- gatecore (SCAIGWY, beta): kurumun kendi AI ajanlarını ServiceCore'a
  bağlayan resmî kapı — kimlikli, yetki kapsamlı, denetlenebilir, maskeli;
  akıllı uçlar AICore eklenti lisanslarıyla sunulur (bypass → tüketim)
- gorevler/ekler/aicore-savunma-stratejisi: savunma stratejisi (md+txt) +
  sözleşme maddeleri taslağı (9 madde: lisans/PoC/partner, hukuk incelemesine)
- CRM listesi: GateCoreAI satırı + ağırlık (32 ürün)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
+++ b/gorevler/ekler/aicore-crm-listesi/AICore_Urun_Listesi_CRM.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -999,128 +999,145 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>GateCoreAI</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Kurumunuzun kendi yapay zekâ ajanlarını ServiceCore'a bağlayan resmî ve denetlenebilir kapı. Kurumun merkezi ajanı (Copilot, Claude, kendi geliştirdiğiniz) ServiceCore'a tek resmî kapıdan bağlanır. Her istek kimlikli, yetki kapsamlı ve denetlenebilir; kişisel veriler ajanlara maskelenerek sunulur. Sayfa: https://www.servicecore.com.tr/aicore/gatecore</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SCAIGWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>— HİZMET VE DESTEK PAKETLERİ —</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>AICORE Launch Ready Paketi</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>AICore eklentileri için anahtar teslim kurulum hizmeti. Yapay zekâ sunucusunun kurulumundan kurumun kendi verisiyle kalibrasyona, ekip eğitiminden gözetimli canlıya alışa kadar uçtan uca devreye alma. Tipik süre 2-4 hafta; sonraki eklentiler aynı altyapıya çok daha hızlı eklenir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-launch-ready</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>SCAILRCP</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AICORE Cloud Ready Paketi</t>
+          <t>AICORE Launch Ready Paketi</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Maskeli Bulut modunda AICore kurulum hizmeti. Kurum ortamına dil modeli kurulmaz; GPU'suz hafif uygulama sunucusu, kişisel verileri denetlenebilir şekilde maskeleyen katman, kalibrasyon ve eğitimle 1-2 haftada devreye alma. Bulut kullanım (token) maliyeti kurumun kendi API hesabına aittir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-cloud-ready</t>
+          <t>AICore eklentileri için anahtar teslim kurulum hizmeti. Yapay zekâ sunucusunun kurulumundan kurumun kendi verisiyle kalibrasyona, ekip eğitiminden gözetimli canlıya alışa kadar uçtan uca devreye alma. Tipik süre 2-4 hafta; sonraki eklentiler aynı altyapıya çok daha hızlı eklenir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-launch-ready</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SCAICRCP</t>
+          <t>SCAILRCP</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AICORE Quick Start Konfigürasyon Paketi</t>
+          <t>AICORE Cloud Ready Paketi</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Mevcut AICore altyapısına sonraki her eklentinin devreye alma paketi. Altyapı işi tekrarlanmaz: eklenti kurulumu, varsa ek erişimlerin bağlanması, eklentiye özel kalibrasyon, doğrulama setinin genişletilmesi ve odaklı eğitim — tipik 2-5 gün. İlk kurulum Launch Ready/Cloud Ready ile yapılır; sonraki her eklenti Quick Start ile eklenir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-quick-start</t>
+          <t>Maskeli Bulut modunda AICore kurulum hizmeti. Kurum ortamına dil modeli kurulmaz; GPU'suz hafif uygulama sunucusu, kişisel verileri denetlenebilir şekilde maskeleyen katman, kalibrasyon ve eğitimle 1-2 haftada devreye alma. Bulut kullanım (token) maliyeti kurumun kendi API hesabına aittir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-cloud-ready</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SCAIQSCP</t>
+          <t>SCAICRCP</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AICORE Silver Destek Paketi</t>
+          <t>AICORE Quick Start Konfigürasyon Paketi</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>AICore eklentileri için temel yıllık bakım. Yıllık 15 ticket, 5x8 kapsam, sürüm güncellemeleri + güncelleme sonrası otomatik doğrulama, yılda 1 yeniden kalibrasyon ve yıllık sağlık raporu. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>Mevcut AICore altyapısına sonraki her eklentinin devreye alma paketi. Altyapı işi tekrarlanmaz: eklenti kurulumu, varsa ek erişimlerin bağlanması, eklentiye özel kalibrasyon, doğrulama setinin genişletilmesi ve odaklı eğitim — tipik 2-5 gün. İlk kurulum Launch Ready/Cloud Ready ile yapılır; sonraki her eklenti Quick Start ile eklenir. Sayfa: https://www.servicecore.com.tr/hizmetler/setup/aicore-quick-start</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SCAISSP</t>
+          <t>SCAIQSCP</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AICORE Gold Destek Paketi</t>
+          <t>AICORE Silver Destek Paketi</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Birden çok AICore eklentisi kullanan kurumlar için yıllık bakım. Yıllık 30 ticket, 5x8 kapsam + telefon desteği, yılda 2 yeniden kalibrasyon, çeyreklik sağlık raporu ve AI Health-Check. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>AICore eklentileri için temel yıllık bakım. Yıllık 15 ticket, 5x8 kapsam, sürüm güncellemeleri + güncelleme sonrası otomatik doğrulama, yılda 1 yeniden kalibrasyon ve yıllık sağlık raporu. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SCAIGSP</t>
+          <t>SCAISSP</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AICORE Platinum Destek Paketi</t>
+          <t>AICORE Gold Destek Paketi</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Yapay zekâyı iş akışının parçası yapmış kurumlar için yıllık bakım. Yıllık 60 ticket, 7x8 kapsam + anlık mesaj, yılda 4 yeniden kalibrasyon, aylık sağlık raporu, yüksek öncelikli müdahale ve model performansı izleme. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+          <t>Birden çok AICore eklentisi kullanan kurumlar için yıllık bakım. Yıllık 30 ticket, 5x8 kapsam + telefon desteği, yılda 2 yeniden kalibrasyon, çeyreklik sağlık raporu ve AI Health-Check. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SCAIPSP</t>
+          <t>SCAIGSP</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>AICORE Platinum Destek Paketi</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zekâyı iş akışının parçası yapmış kurumlar için yıllık bakım. Yıllık 60 ticket, 7x8 kapsam + anlık mesaj, yılda 4 yeniden kalibrasyon, aylık sağlık raporu, yüksek öncelikli müdahale ve model performansı izleme. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>SCAIPSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>AICORE Mission Critical Destek Paketi</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Yapay zekâsı kesintiye tahammülü olmayan kurumlar için en üst kademe. Yıllık 60 ticket, 7x24 kesintisiz kapsam, sınırsız yeniden kalibrasyon, aylık rapor + dönemsel değerlendirme ve adanmış yapay zekâ uzmanı. Sayfa: https://www.servicecore.com.tr/hizmetler/support/aicore-destek</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>SCAIMCSP</t>
         </is>
@@ -1137,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1406,26 +1423,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RisiCoreAI</t>
+          <t>GateCoreAI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SCAIRSK</t>
+          <t>SCAIGWY</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2.7X</t>
+          <t>2.9X</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -1435,43 +1452,43 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>4.0X</t>
+          <t>3.0X</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Zafiyet verisi güncelleme bakımı sürekli</t>
+          <t>Stratejik kapı ürünü; ajan trafiği yönetimi + maskeleme</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RootCoreAI</t>
+          <t>RisiCoreAI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SCAIRTC</t>
+          <t>SCAIRSK</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2.5X</t>
+          <t>2.7X</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>3.0X</t>
+          <t>4.0X</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1481,30 +1498,30 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Öğrenme döngüsü sürekli izleme/bakım ister</t>
+          <t>Zafiyet verisi güncelleme bakımı sürekli</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>StormCoreAI</t>
+          <t>RootCoreAI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SCAISTM</t>
+          <t>SCAIRTC</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>4</v>
       </c>
       <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
           <t>2.5X</t>
@@ -1512,29 +1529,29 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
           <t>4.0X</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>3.0X</t>
-        </is>
-      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Alarm sistemleri entegrasyonu + tepe hacim</t>
+          <t>Öğrenme döngüsü sürekli izleme/bakım ister</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CallCoreAI</t>
+          <t>StormCoreAI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SCAICLL</t>
+          <t>SCAISTM</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1563,60 +1580,60 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Ses akışı + kayıt depolama</t>
+          <t>Alarm sistemleri entegrasyonu + tepe hacim</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DocCoreAI</t>
+          <t>CallCoreAI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SCAIDOC</t>
+          <t>SCAICLL</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>2.3X</t>
+          <t>2.5X</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
+          <t>4.0X</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
           <t>3.0X</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>3.0X</t>
-        </is>
-      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Doküman kaynak erişimi kurulumu; işleme hattı ortak</t>
+          <t>Ses akışı + kayıt depolama</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ClassifyCoreAI</t>
+          <t>DocCoreAI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SCAICLS</t>
+          <t>SCAIDOC</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1645,19 +1662,19 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Kategori/atama eğitimi + müşteri şemasına uyarlama</t>
+          <t>Doküman kaynak erişimi kurulumu; işleme hattı ortak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PredictCoreAI</t>
+          <t>ClassifyCoreAI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SCAIPRD</t>
+          <t>SCAICLS</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1686,19 +1703,19 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Tahmin kalitesi izleme ister</t>
+          <t>Kategori/atama eğitimi + müşteri şemasına uyarlama</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ReportCoreAI</t>
+          <t>PredictCoreAI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SCAIRPT</t>
+          <t>SCAIPRD</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1708,11 +1725,11 @@
         <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>2.2X</t>
+          <t>2.3X</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1722,75 +1739,75 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>2.0X</t>
+          <t>3.0X</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Yönetici görünürlüğü yüksek; rapor şemasına uyarlama</t>
+          <t>Tahmin kalitesi izleme ister</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ReplyCoreAI</t>
+          <t>ReportCoreAI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SCAIRPL</t>
+          <t>SCAIRPT</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
+          <t>2.2X</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
           <t>2.0X</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>2.0X</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>2.0X</t>
-        </is>
-      </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Yüksek görünür değer; teknik olarak hafif</t>
+          <t>Yönetici görünürlüğü yüksek; rapor şemasına uyarlama</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AssetCoreAI</t>
+          <t>ReplyCoreAI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SCAIAST</t>
+          <t>SCAIRPL</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1799,29 +1816,29 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>3.0X</t>
+          <t>2.0X</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>3.0X</t>
+          <t>2.0X</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Telemetri kaynaklarına bağımlı</t>
+          <t>Yüksek görünür değer; teknik olarak hafif</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ImpactCoreAI</t>
+          <t>AssetCoreAI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SCAIIMP</t>
+          <t>SCAIAST</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1831,11 +1848,11 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>1.9X</t>
+          <t>2.0X</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1845,24 +1862,24 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>2.0X</t>
+          <t>3.0X</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Varlık ilişkisi verisine bağımlı</t>
+          <t>Telemetri kaynaklarına bağımlı</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FlowCoreAI</t>
+          <t>ImpactCoreAI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SCAIFLW</t>
+          <t>SCAIIMP</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1891,19 +1908,19 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Yapılandırma düzeyi yazma; onay akışı şart</t>
+          <t>Varlık ilişkisi verisine bağımlı</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ShiftCoreAI</t>
+          <t>FlowCoreAI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SCAISHF</t>
+          <t>SCAIFLW</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1932,19 +1949,19 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>İK/vardiya verisi entegrasyonu</t>
+          <t>Yapılandırma düzeyi yazma; onay akışı şart</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AuditCoreAI</t>
+          <t>ShiftCoreAI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SCAIAUD</t>
+          <t>SCAISHF</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1973,19 +1990,19 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Periyodik denetim; orta kapsam</t>
+          <t>İK/vardiya verisi entegrasyonu</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BudgetCoreAI</t>
+          <t>AuditCoreAI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SCAIBDG</t>
+          <t>SCAIAUD</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2014,60 +2031,60 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Finans verisi entegrasyonu</t>
+          <t>Periyodik denetim; orta kapsam</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MergeCoreAI</t>
+          <t>BudgetCoreAI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SCAIMRG</t>
+          <t>SCAIBDG</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>1.7X</t>
+          <t>1.9X</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
+          <t>3.0X</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
           <t>2.0X</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>2.0X</t>
-        </is>
-      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Motor hazır; sınırlı yüzey</t>
+          <t>Finans verisi entegrasyonu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PriorityCoreAI</t>
+          <t>MergeCoreAI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SCAIPRI</t>
+          <t>SCAIMRG</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -2096,19 +2113,19 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Dar kapsam, hafif</t>
+          <t>Motor hazır; sınırlı yüzey</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KBCoreAI</t>
+          <t>PriorityCoreAI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SCAIKBC</t>
+          <t>SCAIPRI</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -2137,19 +2154,19 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Bilgi bankası taraması; orta kapsam</t>
+          <t>Dar kapsam, hafif</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VisionCoreAI</t>
+          <t>KBCoreAI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SCAIVSN</t>
+          <t>SCAIKBC</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -2178,19 +2195,19 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Görsel okuma; mevcut yeteneğin ürünleşmesi</t>
+          <t>Bilgi bankası taraması; orta kapsam</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ContractCoreAI</t>
+          <t>VisionCoreAI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SCAICNT</t>
+          <t>SCAIVSN</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -2219,19 +2236,19 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Doküman deposu erişimi; orta</t>
+          <t>Görsel okuma; mevcut yeteneğin ürünleşmesi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ProjectCoreAI</t>
+          <t>ContractCoreAI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SCAIPRJ</t>
+          <t>SCAICNT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -2260,23 +2277,23 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Proje verisi analizi; orta</t>
+          <t>Doküman deposu erişimi; orta</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VendorCoreAI</t>
+          <t>ProjectCoreAI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SCAIVND</t>
+          <t>SCAIPRJ</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
         <v>2</v>
@@ -2286,7 +2303,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>1.3X</t>
+          <t>1.7X</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -2301,19 +2318,19 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Dar kapsam</t>
+          <t>Proje verisi analizi; orta</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CoachCoreAI</t>
+          <t>VendorCoreAI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SCAICCH</t>
+          <t>SCAIVND</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2349,53 +2366,53 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SentimentCoreAI</t>
+          <t>CoachCoreAI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SCAISNT</t>
+          <t>SCAICCH</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>1.0X</t>
+          <t>1.3X</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>1.0X</t>
+          <t>2.0X</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>1.0X</t>
+          <t>2.0X</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Basit analiz; taban ürün</t>
+          <t>Dar kapsam</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ToneCoreAI</t>
+          <t>SentimentCoreAI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SCAITON</t>
+          <t>SCAISNT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2431,12 +2448,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TranslateCoreAI</t>
+          <t>ToneCoreAI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SCAITRN</t>
+          <t>SCAITON</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2465,33 +2482,74 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
+          <t>Basit analiz; taban ürün</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TranslateCoreAI</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SCAITRN</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>1.0X</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
           <t>Basit çeviri katmanı; taban ürün</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>Model — üç ayrı çarpan, üç ayrı fiyat kalemi:</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>· Lisans Çarpanı = (0,5·Değer + 0,3·Kurulum + 0,2·Bakım) / taban → modül lisans fiyatı = lisans tabanı × bu çarpan.</t>
+          <t>Model — üç ayrı çarpan, üç ayrı fiyat kalemi:</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>· Kurulum Hizmeti Çarpanı = Kurulum Zorluğu / taban → modül kurulum bedeli = kurulum tabanı (Launch Ready veya Cloud Ready) × bu çarpan.</t>
+          <t>· Lisans Çarpanı = (0,5·Değer + 0,3·Kurulum + 0,2·Bakım) / taban → modül lisans fiyatı = lisans tabanı × bu çarpan.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>· Kurulum Hizmeti Çarpanı = Kurulum Zorluğu / taban → modül kurulum bedeli = kurulum tabanı (Launch Ready veya Cloud Ready) × bu çarpan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>· Destek Hizmeti Çarpanı = Bakım Zorluğu / taban → modülün yıllık destek payı = destek tabanı (Silver/Gold/Platinum) × bu çarpan; sözleşme tek, fiyat toplamdan.</t>
         </is>

</xml_diff>